<commit_message>
feat: Enhance persona pattern rules and improve UI for knowledge sources
- Added persona pattern rules for different personas (P01, P02, P03) with associated allowed actions and descriptions.
- Introduced a new function `visiblePatterns` to filter patterns based on the selected persona.
- Updated `patternDisplay` function to show appropriate names and descriptions based on the selected pattern and persona.
- Modified the rendering of patterns to utilize the new `visiblePatterns` function.
- Improved the UI for knowledge source selection, including a new toggle control and selected state indication.
- Enhanced CSS styles for source rows and selection controls for better visual feedback.
</commit_message>
<xml_diff>
--- a/oci_ai_factory_final_workbook_corrected.xlsx
+++ b/oci_ai_factory_final_workbook_corrected.xlsx
@@ -1,34 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <sheets>
-    <sheet name="01_README" sheetId="1" r:id="rId1"/>
-    <sheet name="02_Personas" sheetId="2" r:id="rId2"/>
-    <sheet name="03_Agent_Patterns" sheetId="3" r:id="rId3"/>
-    <sheet name="04_Knowledge_Sources" sheetId="4" r:id="rId4"/>
-    <sheet name="05_Persona_Pattern_KB_Map" sheetId="5" r:id="rId5"/>
-    <sheet name="06_Experience_Rules" sheetId="6" r:id="rId6"/>
-    <sheet name="07_Persona_Pattern_Scenarios" sheetId="7" r:id="rId7"/>
-    <sheet name="08_Scenario_QnA" sheetId="8" r:id="rId8"/>
-    <sheet name="09_Sample_Responses" sheetId="9" r:id="rId9"/>
-    <sheet name="10_Blueprint_Map" sheetId="10" r:id="rId10"/>
-    <sheet name="11_Content_Repository_Map" sheetId="11" r:id="rId11"/>
-    <sheet name="12_Leaderboard_Config" sheetId="12" r:id="rId12"/>
+    <sheet name="01_README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="02_Personas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="03_Agent_Patterns" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="04_Knowledge_Sources" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="05_Persona_Pattern_KB_Map" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="06_Experience_Rules" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="07_Persona_Pattern_Scenarios" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="08_Scenario_QnA" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="09_Sample_Responses" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="10_Blueprint_Map" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="11_Content_Repository_Map" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="12_Leaderboard_Config" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
+  <definedNames/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
+      <name val="Calibri"/>
       <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="1">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
   </fills>
   <borders count="1">
@@ -44,16 +47,373 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -105,11 +465,18 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -593,11 +960,18 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1329,11 +1703,18 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1421,11 +1802,18 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1516,11 +1904,18 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1608,11 +2003,18 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2576,12 +2978,796 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>KS26</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>AP01</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Finance SharePoint Portal</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Finance guidance pages and working docs</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Budget approvals, close guidance, and finance FAQs</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Doc/Email/Slack</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>KS27</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>AP01</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Finance Jira Knowledge Base</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Finance issue history and runbooks</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Common invoice, coding, and close process fixes</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Jira</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>KS28</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>AP01</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Finance Email Archive</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Shared finance mailbox examples</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Prior finance responses, exceptions, and approvals</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>KS29</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>AP01</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Finance Policy Repository</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>PDF/DOCX finance policy pack</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Travel, reimbursement, budget, and close policies</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>KS30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>AP01</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Call Center Knowledge Articles</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Support articles and troubleshooting guides</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Customer issue articles, FAQs, and resolution guidance</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>KS31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>AP01</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Call Center Email Archive</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Customer email examples</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Prior complaint callbacks, support replies, and service guidance</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>KS32</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>AP01</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Call Center Slack Handoff Channel</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Support collaboration thread samples</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Urgent handoffs, queue guidance, and escalation clarifications</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Slack</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>KS33</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>AP01</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Call Center Escalation SOP Repository</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Support standard operating procedures</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Step-by-step complaint escalation and triage workflows</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>KS34</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>AP01</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Customer Courtesy Policy Repository</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Customer policy and credit guidance</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Courtesy credit, refund, and customer care policy rules</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>KS35</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>AP02</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Call Center Staffing Dataset</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Support team staffing and queue coverage</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Agent counts, queues, shifts, and team capacity</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>KS36</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>AP02</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Support Hiring Pipeline Dataset</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Call center hiring funnel</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Open roles, candidates, time-to-fill, and hiring stages</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>KS37</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>AP02</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Agent Training Dataset</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Training completion and certification data</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Agent learning assignments, queue certifications, and completion status</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>KS38</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>AP02</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Agent Quality Metrics Dataset</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Quality score and performance data</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>QA scores, resolution quality, and team performance metrics</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>KS39</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>AP03</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>HR Employee Contract Documents</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Employee contract document samples</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Employment contracts, clauses, obligations, and renewal dates</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>PDF/DOCX</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>KS40</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>AP03</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>HR Employee Forms Repository</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Employee forms and declarations</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Employee forms, approvals, dates, and status fields</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>KS41</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>AP03</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>HR Reimbursement Documents</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Employee reimbursement document samples</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Expense and reimbursement documents tied to HR policy categories</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>KS42</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>AP02</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Finance Cost Center Dataset</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Finance cost center and headcount data</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Active employee counts, cost centers, and finance ownership</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>KS43</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>AP02</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Payroll Spend Dataset</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Payroll cost and earning transactions</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Payroll spend by region, pay type, and period</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>KS44</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>AP02</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Workforce Cost Forecast Dataset</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Finance workforce planning forecast</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Planned versus forecast workforce cost by quarter</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>KS45</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>AP02</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Recruiting Cost Pipeline Dataset</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Hiring pipeline cost analytics</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Hiring-stage cost impact and finance planning data</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>KS46</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>AP02</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Bonus Performance Dataset</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Performance-linked compensation data</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Bonus spend by rating band and performance outcome</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2816,7 +4002,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>KS15</t>
+          <t>KS39</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2838,7 +4024,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>KS18</t>
+          <t>KS40</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2860,7 +4046,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>KS19</t>
+          <t>KS41</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2948,7 +4134,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>KS02</t>
+          <t>KS26</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2970,7 +4156,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>KS03</t>
+          <t>KS27</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2992,7 +4178,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>KS04</t>
+          <t>KS28</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -3014,7 +4200,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>KS07</t>
+          <t>KS29</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -3036,7 +4222,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>KS08</t>
+          <t>KS42</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -3058,7 +4244,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>KS09</t>
+          <t>KS43</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -3080,7 +4266,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>KS10</t>
+          <t>KS44</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -3102,7 +4288,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>KS11</t>
+          <t>KS45</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -3124,7 +4310,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>KS13</t>
+          <t>KS46</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -3322,7 +4508,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>KS03</t>
+          <t>KS30</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -3344,7 +4530,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>KS04</t>
+          <t>KS31</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -3366,7 +4552,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>KS05</t>
+          <t>KS32</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -3388,7 +4574,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>KS06</t>
+          <t>KS33</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -3410,7 +4596,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>KS07</t>
+          <t>KS34</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -3432,7 +4618,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>KS08</t>
+          <t>KS35</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -3454,7 +4640,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>KS11</t>
+          <t>KS36</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -3476,7 +4662,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>KS12</t>
+          <t>KS37</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -3498,7 +4684,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>KS13</t>
+          <t>KS38</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -3728,11 +4914,18 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -3831,11 +5024,18 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -4319,11 +5519,18 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -5028,17 +6235,17 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>KS15</t>
+          <t>KS39</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Contract Repository</t>
+          <t>HR Employee Contract Documents</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>KS15</t>
+          <t>KS39</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -5095,17 +6302,17 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>KS18</t>
+          <t>KS40</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Employee Forms</t>
+          <t>HR Employee Forms Repository</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>KS18</t>
+          <t>KS40</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -5162,17 +6369,17 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>KS19</t>
+          <t>KS41</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Expense Reports</t>
+          <t>HR Reimbursement Documents</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>KS19</t>
+          <t>KS41</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -5430,17 +6637,17 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>KS02</t>
+          <t>KS26</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>HR SharePoint Portal</t>
+          <t>Finance SharePoint Portal</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>KS02</t>
+          <t>KS26</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -5497,17 +6704,17 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>KS03</t>
+          <t>KS27</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>HR Jira Knowledge Base</t>
+          <t>Finance Jira Knowledge Base</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>KS03</t>
+          <t>KS27</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -5564,17 +6771,17 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>KS04</t>
+          <t>KS28</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>HR Email Archive</t>
+          <t>Finance Email Archive</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>KS04</t>
+          <t>KS28</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -5631,17 +6838,17 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>KS07</t>
+          <t>KS29</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Employee Handbook</t>
+          <t>Finance Policy Repository</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>KS07</t>
+          <t>KS29</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -5698,17 +6905,17 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>KS08</t>
+          <t>KS42</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Employee Master Dataset</t>
+          <t>Finance Cost Center Dataset</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>KS08</t>
+          <t>KS42</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -5765,17 +6972,17 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>KS09</t>
+          <t>KS43</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Payroll Dataset</t>
+          <t>Payroll Spend Dataset</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>KS09</t>
+          <t>KS43</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -5832,17 +7039,17 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>KS10</t>
+          <t>KS44</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Workforce Planning Dataset</t>
+          <t>Workforce Cost Forecast Dataset</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>KS10</t>
+          <t>KS44</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -5899,17 +7106,17 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>KS11</t>
+          <t>KS45</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Recruiting Analytics Dataset</t>
+          <t>Recruiting Cost Pipeline Dataset</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>KS11</t>
+          <t>KS45</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -5966,17 +7173,17 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>KS13</t>
+          <t>KS46</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Performance Dataset</t>
+          <t>Bonus Performance Dataset</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>KS13</t>
+          <t>KS46</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -6569,17 +7776,17 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>KS03</t>
+          <t>KS30</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>HR Jira Knowledge Base</t>
+          <t>Call Center Knowledge Articles</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>KS03</t>
+          <t>KS30</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -6636,17 +7843,17 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>KS04</t>
+          <t>KS31</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>HR Email Archive</t>
+          <t>Call Center Email Archive</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>KS04</t>
+          <t>KS31</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -6703,17 +7910,17 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>KS05</t>
+          <t>KS32</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>HR Slack Channel</t>
+          <t>Call Center Slack Handoff Channel</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>KS05</t>
+          <t>KS32</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -6770,17 +7977,17 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>KS06</t>
+          <t>KS33</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>HR SOP Repository</t>
+          <t>Call Center Escalation SOP Repository</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>KS06</t>
+          <t>KS33</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -6837,17 +8044,17 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>KS07</t>
+          <t>KS34</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Employee Handbook</t>
+          <t>Customer Courtesy Policy Repository</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>KS07</t>
+          <t>KS34</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -6904,17 +8111,17 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>KS08</t>
+          <t>KS35</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Employee Master Dataset</t>
+          <t>Call Center Staffing Dataset</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>KS08</t>
+          <t>KS35</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -6971,17 +8178,17 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>KS11</t>
+          <t>KS36</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Recruiting Analytics Dataset</t>
+          <t>Support Hiring Pipeline Dataset</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>KS11</t>
+          <t>KS36</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -7038,17 +8245,17 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>KS12</t>
+          <t>KS37</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Learning Dataset</t>
+          <t>Agent Training Dataset</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>KS12</t>
+          <t>KS37</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -7105,17 +8312,17 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>KS13</t>
+          <t>KS38</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Performance Dataset</t>
+          <t>Agent Quality Metrics Dataset</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>KS13</t>
+          <t>KS38</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -7810,11 +9017,18 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -8294,17 +9508,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>KS15</t>
+          <t>KS39</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Contract Repository</t>
+          <t>HR Employee Contract Documents</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>KS15</t>
+          <t>KS39</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -8341,17 +9555,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>KS18</t>
+          <t>KS40</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Employee Forms</t>
+          <t>HR Employee Forms Repository</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>KS18</t>
+          <t>KS40</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -8388,17 +9602,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>KS19</t>
+          <t>KS41</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Expense Reports</t>
+          <t>HR Reimbursement Documents</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>KS19</t>
+          <t>KS41</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -8576,17 +9790,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>KS02</t>
+          <t>KS26</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>HR SharePoint Portal</t>
+          <t>Finance SharePoint Portal</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>KS02</t>
+          <t>KS26</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -8623,17 +9837,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>KS03</t>
+          <t>KS27</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>HR Jira Knowledge Base</t>
+          <t>Finance Jira Knowledge Base</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>KS03</t>
+          <t>KS27</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -8670,17 +9884,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>KS04</t>
+          <t>KS28</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>HR Email Archive</t>
+          <t>Finance Email Archive</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>KS04</t>
+          <t>KS28</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -8717,17 +9931,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>KS07</t>
+          <t>KS29</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Employee Handbook</t>
+          <t>Finance Policy Repository</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>KS07</t>
+          <t>KS29</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -8764,17 +9978,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>KS08</t>
+          <t>KS42</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Employee Master Dataset</t>
+          <t>Finance Cost Center Dataset</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>KS08</t>
+          <t>KS42</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -8811,17 +10025,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>KS09</t>
+          <t>KS43</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Payroll Dataset</t>
+          <t>Payroll Spend Dataset</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>KS09</t>
+          <t>KS43</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -8858,17 +10072,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>KS10</t>
+          <t>KS44</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Workforce Planning Dataset</t>
+          <t>Workforce Cost Forecast Dataset</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>KS10</t>
+          <t>KS44</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -8905,17 +10119,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>KS11</t>
+          <t>KS45</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Recruiting Analytics Dataset</t>
+          <t>Recruiting Cost Pipeline Dataset</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>KS11</t>
+          <t>KS45</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -8952,17 +10166,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>KS13</t>
+          <t>KS46</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Performance Dataset</t>
+          <t>Bonus Performance Dataset</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>KS13</t>
+          <t>KS46</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -9375,17 +10589,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>KS03</t>
+          <t>KS30</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>HR Jira Knowledge Base</t>
+          <t>Call Center Knowledge Articles</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>KS03</t>
+          <t>KS30</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -9422,17 +10636,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>KS04</t>
+          <t>KS31</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>HR Email Archive</t>
+          <t>Call Center Email Archive</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>KS04</t>
+          <t>KS31</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -9469,17 +10683,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>KS05</t>
+          <t>KS32</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>HR Slack Channel</t>
+          <t>Call Center Slack Handoff Channel</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>KS05</t>
+          <t>KS32</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -9516,17 +10730,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>KS06</t>
+          <t>KS33</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>HR SOP Repository</t>
+          <t>Call Center Escalation SOP Repository</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>KS06</t>
+          <t>KS33</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -9563,17 +10777,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>KS07</t>
+          <t>KS34</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Employee Handbook</t>
+          <t>Customer Courtesy Policy Repository</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>KS07</t>
+          <t>KS34</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -9610,17 +10824,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>KS08</t>
+          <t>KS35</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Employee Master Dataset</t>
+          <t>Call Center Staffing Dataset</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>KS08</t>
+          <t>KS35</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -9657,17 +10871,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>KS11</t>
+          <t>KS36</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Recruiting Analytics Dataset</t>
+          <t>Support Hiring Pipeline Dataset</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>KS11</t>
+          <t>KS36</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -9704,17 +10918,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>KS12</t>
+          <t>KS37</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Learning Dataset</t>
+          <t>Agent Training Dataset</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>KS12</t>
+          <t>KS37</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -9751,17 +10965,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>KS13</t>
+          <t>KS38</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Performance Dataset</t>
+          <t>Agent Quality Metrics Dataset</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>KS13</t>
+          <t>KS38</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -10261,5 +11475,6 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>